<commit_message>
[feat] MatchRuleData 랭킹별 라운드 조건 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/MatchRuleData.xlsx
+++ b/JsonConverter/ExcelFiles/MatchRuleData.xlsx
@@ -19,28 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
-  <x:si>
-    <x:t>5라운드 경기</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>float</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3라운드 경기</x:t>
-  </x:si>
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
   <x:si>
     <x:t>int</x:t>
   </x:si>
@@ -51,16 +30,52 @@
     <x:t>RoundBreakSeconds</x:t>
   </x:si>
   <x:si>
+    <x:t>IncludeChampion</x:t>
+  </x:si>
+  <x:si>
     <x:t>RoundCount</x:t>
+  </x:si>
+  <x:si>
+    <x:t>bool</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3라운드 경기</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5라운드 경기</x:t>
+  </x:si>
+  <x:si>
+    <x:t>float</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IncludeUnranked</x:t>
+  </x:si>
+  <x:si>
+    <x:t>rule_round_5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MaxOpponentRank</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RoundSeconds</x:t>
   </x:si>
   <x:si>
     <x:t>rule_round_3</x:t>
   </x:si>
   <x:si>
-    <x:t>RoundSeconds</x:t>
-  </x:si>
-  <x:si>
-    <x:t>rule_round_5</x:t>
+    <x:t>MinOpponentRank</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -831,64 +846,88 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:H35"/>
+  <x:dimension ref="A1:I35"/>
   <x:sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="25.4296875" style="1" customWidth="1"/>
     <x:col min="2" max="2" width="19.54296875" style="1" customWidth="1"/>
     <x:col min="3" max="3" width="41.5703125" style="1" customWidth="1"/>
     <x:col min="4" max="6" width="20.26953125" style="1" customWidth="1"/>
-    <x:col min="7" max="7" width="30.54296875" style="1" customWidth="1"/>
-    <x:col min="8" max="8" width="26.54296875" style="1" customWidth="1"/>
-    <x:col min="9" max="9" width="20" style="1" customWidth="1"/>
-    <x:col min="10" max="12" width="12.54296875" style="1" bestFit="1" customWidth="1"/>
-    <x:col min="13" max="13" width="15.71484375" style="1" customWidth="1"/>
-    <x:col min="14" max="14" width="17.4296875" style="1" customWidth="1"/>
-    <x:col min="15" max="16384" width="12.54296875" style="1"/>
+    <x:col min="7" max="8" width="30.54296875" style="1" customWidth="1"/>
+    <x:col min="9" max="9" width="26.54296875" style="1" customWidth="1"/>
+    <x:col min="10" max="10" width="20" style="1" customWidth="1"/>
+    <x:col min="11" max="13" width="12.54296875" style="1" bestFit="1" customWidth="1"/>
+    <x:col min="14" max="14" width="15.71484375" style="1" customWidth="1"/>
+    <x:col min="15" max="15" width="17.4296875" style="1" customWidth="1"/>
+    <x:col min="16" max="16384" width="12.54296875" style="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:1" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:9" ht="13.199999999999999">
+      <x:c r="A2" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H2" s="1" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I2" s="1" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:9" s="7" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A3" s="2" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C3" s="7" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D3" s="7" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E3" s="7" t="s">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:5" ht="13.199999999999999">
-      <x:c r="A2" s="1" t="s">
+      <x:c r="F3" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G3" s="7" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H3" s="7" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B2" s="1" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C2" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="E2" s="1" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:5" s="7" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A3" s="2" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B3" s="2" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C3" s="7" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D3" s="7" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="E3" s="7" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:8" ht="15.75" customHeight="1">
+      <x:c r="I3" s="7" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:9" ht="15.75" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>11</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
         <x:v>6</x:v>
@@ -902,14 +941,25 @@
       <x:c r="E4" s="1">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="H4" s="4"/>
-    </x:row>
-    <x:row r="5" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F4" s="1">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G4" s="1">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H4" s="1" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I4" s="4" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:9" ht="15.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>0</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C5" s="1">
         <x:v>5</x:v>
@@ -919,6 +969,18 @@
       </x:c>
       <x:c r="E5" s="1">
         <x:v>10</x:v>
+      </x:c>
+      <x:c r="F5" s="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G5" s="1">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H5" s="1" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I5" s="1" t="b">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:2" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
[feat] MatchRuleData 전투 행동 실행 간격 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/MatchRuleData.xlsx
+++ b/JsonConverter/ExcelFiles/MatchRuleData.xlsx
@@ -19,51 +19,42 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
   <x:si>
-    <x:t>int</x:t>
+    <x:t>RoundCount</x:t>
   </x:si>
   <x:si>
     <x:t>Id</x:t>
   </x:si>
   <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
     <x:t>RoundBreakSeconds</x:t>
   </x:si>
   <x:si>
-    <x:t>RoundCount</x:t>
+    <x:t>고유 ID</x:t>
   </x:si>
   <x:si>
     <x:t>3라운드 경기</x:t>
   </x:si>
   <x:si>
-    <x:t>bool</x:t>
+    <x:t>5라운드 경기</x:t>
   </x:si>
   <x:si>
-    <x:t>5라운드 경기</x:t>
+    <x:t>string</x:t>
   </x:si>
   <x:si>
     <x:t>Name</x:t>
   </x:si>
   <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>float</x:t>
+    <x:t>bool</x:t>
   </x:si>
   <x:si>
     <x:t>(name)</x:t>
   </x:si>
   <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RoundSeconds</x:t>
-  </x:si>
-  <x:si>
-    <x:t>rule_round_3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MinOpponentRank</x:t>
+    <x:t>float</x:t>
   </x:si>
   <x:si>
     <x:t>MaxOpponentRank</x:t>
@@ -72,10 +63,22 @@
     <x:t>IncludeUnranked</x:t>
   </x:si>
   <x:si>
+    <x:t>rule_round_5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MinOpponentRank</x:t>
+  </x:si>
+  <x:si>
     <x:t>IncludeChampion</x:t>
   </x:si>
   <x:si>
-    <x:t>rule_round_5</x:t>
+    <x:t>rule_round_3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RoundSeconds</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ActionIntervalSeconds</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -846,91 +849,97 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:I35"/>
+  <x:dimension ref="A1:J35"/>
   <x:sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="25.4296875" style="1" customWidth="1"/>
     <x:col min="2" max="2" width="19.54296875" style="1" customWidth="1"/>
     <x:col min="3" max="3" width="41.5703125" style="1" customWidth="1"/>
-    <x:col min="4" max="6" width="20.26953125" style="1" customWidth="1"/>
-    <x:col min="7" max="8" width="30.54296875" style="1" customWidth="1"/>
-    <x:col min="9" max="9" width="26.54296875" style="1" customWidth="1"/>
-    <x:col min="10" max="10" width="20" style="1" customWidth="1"/>
-    <x:col min="11" max="13" width="12.54296875" style="1" bestFit="1" customWidth="1"/>
-    <x:col min="14" max="14" width="15.71484375" style="1" customWidth="1"/>
-    <x:col min="15" max="15" width="17.4296875" style="1" customWidth="1"/>
-    <x:col min="16" max="16384" width="12.54296875" style="1"/>
+    <x:col min="4" max="7" width="20.26953125" style="1" customWidth="1"/>
+    <x:col min="8" max="9" width="30.54296875" style="1" customWidth="1"/>
+    <x:col min="10" max="10" width="26.54296875" style="1" customWidth="1"/>
+    <x:col min="11" max="11" width="20" style="1" customWidth="1"/>
+    <x:col min="12" max="14" width="12.54296875" style="1" bestFit="1" customWidth="1"/>
+    <x:col min="15" max="15" width="15.71484375" style="1" customWidth="1"/>
+    <x:col min="16" max="16" width="17.4296875" style="1" customWidth="1"/>
+    <x:col min="17" max="16384" width="12.54296875" style="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:1" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:9" ht="13.199999999999999">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:10" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I2" s="1" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E2" s="1" t="s">
+      <x:c r="J2" s="1" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="F2" s="1" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G2" s="1" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H2" s="1" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="I2" s="1" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:9" s="7" customFormat="1" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="3" spans="1:10" s="7" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="2" t="s">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C3" s="7" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D3" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E3" s="7" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D3" s="7" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="E3" s="7" t="s">
-        <x:v>2</x:v>
-      </x:c>
       <x:c r="F3" s="7" t="s">
-        <x:v>14</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G3" s="7" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="H3" s="7" t="s">
-        <x:v>17</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="I3" s="7" t="s">
         <x:v>16</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" spans="1:9" ht="15.75" customHeight="1">
+      <x:c r="J3" s="7" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:10" ht="15.75" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>13</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C4" s="1">
         <x:v>3</x:v>
@@ -942,21 +951,24 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="F4" s="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G4" s="1">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="G4" s="1">
+      <x:c r="H4" s="1">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="H4" s="1" t="b">
+      <x:c r="I4" s="1" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I4" s="4" t="b">
+      <x:c r="J4" s="4" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" spans="1:9" ht="15.75" customHeight="1">
+    <x:row r="5" spans="1:10" ht="15.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
-        <x:v>18</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
         <x:v>6</x:v>
@@ -974,12 +986,15 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H5" s="1">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H5" s="1" t="b">
+      <x:c r="I5" s="1" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I5" s="1" t="b">
+      <x:c r="J5" s="1" t="b">
         <x:v>0</x:v>
       </x:c>
     </x:row>

</xml_diff>